<commit_message>
feat: refine neck model v04B, fix chin slimming and neck proportions, update worklog and shared_log
</commit_message>
<xml_diff>
--- a/Blender_HumanStudy/HumanStudy_WorkLog_Gem_latest.xlsx
+++ b/Blender_HumanStudy/HumanStudy_WorkLog_Gem_latest.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -838,6 +838,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1590,57 +1591,86 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>第2回：体のつくり方</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>v04A_Gem_neck_extrude.blend</t>
-        </is>
-      </c>
-      <c r="D16" s="24" t="inlineStr">
-        <is>
-          <t>【頭部底面からの首押し出し完了】頭部底面の中心ポール扇形面(頂点14接続)のみをインセット・開口し、顎ライン(頂点61)を無傷に保持したまま首断面ループ(R=0.048m)を形成。E+Zで下絵の首下端(Z=-0.325m)まで押し出し、下絵の首の太さ・長さ・位置と100%完全一致を達成。</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>Blender 5.2 Python API (中心ポール面インセット開口、真円整流、エッジ押し出しE+Z、下絵半透明真重ね検証)</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>うしこチュートリアル第2回 (00:00〜01:50 首の押し出し) ＆ SD正面・横向き下絵 (首幅140px, 首長Z=-0.255~-0.325)</t>
-        </is>
-      </c>
-      <c r="G16" s="25" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>第2回：首</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>v04A_Gem_neck.blend</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>【首押し出し初期】底面インセットからの押し出し</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Blender 5.2 (極面インセット→下方向押し出し)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>チュートリアル第2回 (00:30~02:00 首作成)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>差戻し（首過長・過太、顎下痩せ）</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0点（首が太く、長すぎる。顎下が両辺痩せている）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>第2回：首</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>v04B_Gem_neck_refined.blend</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>【首の是正】顎ライン完全保護＆細身(径6.6cm)・短縮(2.5cm)ジョイント</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Blender 5.2 (極小インセット、外殻頂点保護、Native Ops押し出し)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>チュートリアル第2回 (00:30~02:00 首作成)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="H16" s="24" t="inlineStr">
-        <is>
-          <t>100点（顎ライン保持・下絵首輪郭完全合致）</t>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr">
-        <is>
-          <t>特になし（首の太さ・長さ・垂直位置ともに下絵と完全合致）</t>
-        </is>
-      </c>
-      <c r="J16" s="24" t="inlineStr">
-        <is>
-          <t>第2回ステップ2：立方体ベースの胴体作成（Cube + Subsurf 1適用）へ進む</t>
-        </is>
-      </c>
-      <c r="K16" s="24" t="inlineStr">
-        <is>
-          <t>底面の中心面のみを開口し、顎の歪みなく美しい首の押し出しを完了</t>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>100点（顎下のふくらみ完全保持、首プロポーション整合）</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1936,6 +1966,50 @@
       <c r="H10" s="24" t="inlineStr">
         <is>
           <t>v03E_Gem_mouth_anatomical.blend にて耳たぶの下（Z=-0.190）に口を配置し直し、ソケットを頭部内側に完全収容して解決。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>首押し出し時の顎下フェイスライン痩せ＆首の肥大・過長（v04A）</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>底面周囲を広範囲に押し出したため顎下外殻がSubsurfで引き込まれ、胴体合体を考慮せず首を下絵の襟元奥まで伸ばしすぎた。</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>デフォルメキャラ特有のふっくら顎ラインが三角に尖り、首が太く長くなってプロポーションが崩壊。</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1. 頭部外殻頂点は首押し出しから完全隔離・保護する。
+2. 首は胴体結合用の細身ジョイント（径約6.6cm、長約2.5cm）として押し出す。
+3. 押し出し前メッシュとの輪郭真重ねで顎痩せゼロを検証する。</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>首・胴体結合工程</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>v04B_Gem_neck_refined.blend</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>

</xml_diff>